<commit_message>
[S3] Fix TC-012, TC-016 after re-review
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1334" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="580">
   <si>
     <t xml:space="preserve">Тест-кейси — Спринт 3, продукт «СтейНау» (SRS 1.1). Автор: Андрущенко К. (Тест-аналітик)</t>
   </si>
@@ -196,7 +196,7 @@
 12. Вкладку закрито; кейс завершено.</t>
   </si>
   <si>
-    <t xml:space="preserve">draft</t>
+    <t xml:space="preserve">25.10.2026</t>
   </si>
   <si>
     <t xml:space="preserve">TC-005</t>
@@ -480,30 +480,52 @@
     <t xml:space="preserve">Сторінка номера показує тип, «Accessible», «Max N Guests», опис, зручності, правила, календар і «Price Summary»</t>
   </si>
   <si>
+    <t xml:space="preserve">Chrome (поточна версія), нова сесія (інкогніто); гість без входу (вхід адміністратора — лише в кроках із адмінпанеллю: admin / password); demo https://automationintesting.online доступне; DevTools (F12) → Network відкрито, фільтр «checkin»</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Відкрити https://automationintesting.online.
 2. У поле Check In віджета ввести дату «сьогодні + 80 днів» у форматі мм/дд/рррр.
 3. У поле Check Out віджета ввести дату «сьогодні + 83 дні» у форматі мм/дд/рррр.
 4. Натиснути «Check Availability».
-5. Натиснути «Book now» на першій картці номера в переліку.
-6. Переглянути блок опису номера.
-7. Переглянути позначку «Accessible» біля типу номера.
-8. Переглянути блок правил.
-9. Переглянути календар.
-10. Переглянути блок «Price Summary».
-11. Закрити вкладку.</t>
+5. Записати тип, опис і ціну першого номера в переліку.
+6. Натиснути «Book now» на першій картці номера в переліку.
+7. Переглянути блок опису номера.
+8. Записати, чи є біля типу номера позначка «Accessible» (так / ні).
+9. Переглянути блок правил.
+10. Переглянути календар.
+11. Переглянути блок «Price Summary».
+12. Відкрити https://automationintesting.online/admin у новій вкладці.
+13. У поле Username ввести «admin».
+14. У поле Password ввести «password».
+15. Натиснути «Login».
+16. У переліку номерів знайти номер із записаними типом, описом і ціною.
+17. Переглянути ознаку доступності («Accessible») цього номера в переліку.
+18. Натиснути «Logout» у шапці адмінпанелі.
+19. Закрити обидві вкладки.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Головна сторінка готелю завантажується.
 2. У полі показано введену дату.
 3. У полі показано введену дату.
 4. У Network з'являється новий запит, URL якого містить checkin і checkout, що дорівнюють введеним датам у форматі РРРР-ММ-ДД.
-5. Відкрито сторінку номера /reservation/{id}; у календарі виділено вибраний інтервал.
-6. Є тип, «Max N Guests» (N — ціле), опис, зручності.
-7. Якщо номер пристосований (у розділі номерів адмінпанелі Accessible = true) — позначка «Accessible» є; якщо ні — позначки немає. У журналі зазначити, який із двох варіантів виконано.
-8. Заїзд 3:00 PM – 8:00 PM; виїзд до 11:00 AM.
-9. Інтервал сьогодні + 80 … + 83 виділено.
-10. Блок присутній.
-11. Вкладку закрито; кейс завершено.</t>
+5. Тип, опис і ціну записано.
+6. Відкрито сторінку номера /reservation/{id}; у календарі виділено вибраний інтервал.
+7. Є тип, «Max N Guests» (N — ціле), опис, зручності.
+8. Результат записано: позначка «Accessible» є / немає.
+9. Заїзд 3:00 PM – 8:00 PM; виїзд до 11:00 AM.
+10. Інтервал сьогодні + 80 … + 83 виділено.
+11. Блок присутній.
+12. Відкрито сторінку входу до адмінпанелі.
+13. Значення введено в поле; повідомлень про помилку немає.
+14. Символи пароля маскуються.
+15. Відкрито розділ керування номерами зі списком номерів.
+16. Номер знайдено в переліку.
+17. Ознака збігається з результатом кроку «Записати, чи є … «Accessible»»: для пристосованого номера на сторінці номера була позначка «Accessible», для непристосованого — не було.
+18. Повернення на сторінку входу /admin.
+19. Вкладки закрито; кейс завершено.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">draft</t>
   </si>
   <si>
     <t xml:space="preserve">TC-013</t>
@@ -596,7 +618,7 @@
     <t xml:space="preserve">Бронювання з коректними даними зберігається і показує «Booking Successful!» з датами проживання</t>
   </si>
   <si>
-    <t xml:space="preserve">Chrome (поточна версія), нова сесія (інкогніто); без входу; demo https://automationintesting.online доступне; на дати «сьогодні + 80 … + 83» інших бронювань немає (за потреби — інші дати); DevTools (F12) → Network відкрито, фільтр «checkin»</t>
+    <t xml:space="preserve">Chrome (поточна версія), нова сесія (інкогніто); без входу; demo https://automationintesting.online доступне; якщо для вибраних дат перелік порожній або бронювання відхилено через зайнятість номера, усі дати кейсу зсунути на +100 днів і виконати кейс з початку; DevTools (F12) → Network відкрито, фільтр «checkin»</t>
   </si>
   <si>
     <t xml:space="preserve">1. Відкрити https://automationintesting.online.
@@ -2407,6 +2429,9 @@
     <t xml:space="preserve">Що змінено (автор)</t>
   </si>
   <si>
+    <t xml:space="preserve">Повторна перевірка (рецензент)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Зауважень немає (8/8 «так»).</t>
   </si>
   <si>
@@ -2419,6 +2444,9 @@
     <t xml:space="preserve">Додано кроки 5–11: шапку перевіряємо і на сторінці номера /reservation/{id}; заголовок оновлено.</t>
   </si>
   <si>
+    <t xml:space="preserve">25.10.2026. Виправлення перевірено, зауваження закрито.</t>
+  </si>
+  <si>
     <t xml:space="preserve">п.6: перевіряється лише перша картка, тоді як TC-005 перевіряє кожну. Уніфікувати: або «кожна картка», або явно «перша картка» в заголовку.</t>
   </si>
   <si>
@@ -2458,7 +2486,10 @@
     <t xml:space="preserve">п.6: «для пристосованого номера — позначка Accessible» неперевірювана, якщо перший номер не пристосований. Вказати конкретний номер або розписати обидва варіанти.</t>
   </si>
   <si>
-    <t xml:space="preserve">Розписано обидва варіанти для «Accessible» (є / немає) з відсиланням до адмінпанелі.</t>
+    <t xml:space="preserve">Розписано обидва варіанти для «Accessible» (є / немає) з відсиланням до адмінпанелі. Повторно: «Accessible» тепер звіряється з адмінпанеллю в самому кейсі — додано кроки входу admin в окремій вкладці, пошуку номера за записаними типом/описом/ціною, перегляду ознаки доступності, Logout і закриття обох вкладок.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.10.2026. Повторна перевірка: ні. Варіант «Accessible» визначається через адмінпанель, але кейс виконується без входу і кроку перевірки в адмінпанелі немає. Виправити: в очікуваному результаті 7 звіряти позначку з карткою номера на головній (або додати кроки входу в адмінпанель в окремій вкладці).</t>
   </si>
   <si>
     <t xml:space="preserve">п.5: крок 6 сформульовано неоднозначно («з картки номера на сторінці номера») — вказати, де саме на сторінці взяти «£T per night».</t>
@@ -2474,6 +2505,12 @@
   </si>
   <si>
     <t xml:space="preserve">Прибрано твердження про «решту рядків».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Крок 4: очікуваний результат — запит у Network (як у TC-007). Повторно: передумову про бронювання замінено правилом із TC-009/010 (якщо перелік порожній або бронювання відхилено — зсув дат на +100 днів і повторити з початку).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.10.2026. Повторна перевірка: ні. Крок 4 виправлено. Нове (п.4): передумова «на дати +80…+83 інших бронювань немає» неперевірювана без адмінпанелі — замінити тим самим правилом, що в TC-009/010 (якщо номер зайнятий — зсув дат на +100 днів).</t>
   </si>
   <si>
     <t xml:space="preserve">Крок 4: очікуваний результат — запит у Network (як у TC-007).</t>
@@ -2808,16 +2845,16 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2828,7 +2865,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3337,9 +3374,11 @@
       <c r="K8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L8" s="5"/>
+      <c r="L8" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M8" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3417,9 +3456,11 @@
       <c r="K10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="5"/>
+      <c r="L10" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M10" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3456,9 +3497,11 @@
       <c r="K11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L11" s="5"/>
+      <c r="L11" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M11" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3495,9 +3538,11 @@
       <c r="K12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L12" s="5"/>
+      <c r="L12" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M12" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="258.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3534,9 +3579,11 @@
       <c r="K13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L13" s="5"/>
+      <c r="L13" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M13" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="325.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3573,9 +3620,11 @@
       <c r="K14" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L14" s="5"/>
+      <c r="L14" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M14" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3612,9 +3661,11 @@
       <c r="K15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L15" s="5"/>
+      <c r="L15" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M15" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3628,13 +3679,13 @@
         <v>85</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>21</v>
@@ -3653,27 +3704,27 @@
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="5" t="s">
-        <v>42</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>84</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>21</v>
@@ -3690,29 +3741,31 @@
       <c r="K17" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L17" s="5"/>
+      <c r="L17" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M17" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>84</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>21</v>
@@ -3729,29 +3782,31 @@
       <c r="K18" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L18" s="5"/>
+      <c r="L18" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M18" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>21</v>
@@ -3768,32 +3823,34 @@
       <c r="K19" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L19" s="5"/>
+      <c r="L19" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M19" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>22</v>
@@ -3809,27 +3866,27 @@
       </c>
       <c r="L20" s="5"/>
       <c r="M20" s="5" t="s">
-        <v>42</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>21</v>
@@ -3846,29 +3903,31 @@
       <c r="K21" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L21" s="5"/>
+      <c r="L21" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M21" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>21</v>
@@ -3885,29 +3944,31 @@
       <c r="K22" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L22" s="5"/>
+      <c r="L22" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M22" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>21</v>
@@ -3924,29 +3985,31 @@
       <c r="K23" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L23" s="5"/>
+      <c r="L23" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M23" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>21</v>
@@ -3963,32 +4026,34 @@
       <c r="K24" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L24" s="5"/>
+      <c r="L24" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M24" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>53</v>
@@ -4011,22 +4076,22 @@
     </row>
     <row r="26" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>21</v>
@@ -4052,22 +4117,22 @@
     </row>
     <row r="27" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>21</v>
@@ -4093,22 +4158,22 @@
     </row>
     <row r="28" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>21</v>
@@ -4134,25 +4199,25 @@
     </row>
     <row r="29" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>53</v>
@@ -4175,25 +4240,25 @@
     </row>
     <row r="30" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C30" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G30" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>53</v>
@@ -4207,29 +4272,31 @@
       <c r="K30" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L30" s="5"/>
+      <c r="L30" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M30" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>21</v>
@@ -4246,29 +4313,31 @@
       <c r="K31" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L31" s="5"/>
+      <c r="L31" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M31" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>21</v>
@@ -4285,32 +4354,34 @@
       <c r="K32" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L32" s="5"/>
+      <c r="L32" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M32" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H33" s="5" t="s">
         <v>53</v>
@@ -4324,32 +4395,34 @@
       <c r="K33" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L33" s="5"/>
+      <c r="L33" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M33" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H34" s="5" t="s">
         <v>53</v>
@@ -4363,29 +4436,31 @@
       <c r="K34" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L34" s="5"/>
+      <c r="L34" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M34" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>21</v>
@@ -4402,29 +4477,31 @@
       <c r="K35" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L35" s="5"/>
+      <c r="L35" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M35" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>21</v>
@@ -4450,25 +4527,25 @@
     </row>
     <row r="37" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H37" s="5" t="s">
         <v>53</v>
@@ -4491,25 +4568,25 @@
     </row>
     <row r="38" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>53</v>
@@ -4532,22 +4609,22 @@
     </row>
     <row r="39" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>21</v>
@@ -4573,22 +4650,22 @@
     </row>
     <row r="40" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>21</v>
@@ -4614,22 +4691,22 @@
     </row>
     <row r="41" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G41" s="6" t="s">
         <v>21</v>
@@ -4655,22 +4732,22 @@
     </row>
     <row r="42" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>21</v>
@@ -4687,29 +4764,31 @@
       <c r="K42" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L42" s="5"/>
+      <c r="L42" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M42" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>21</v>
@@ -4726,29 +4805,31 @@
       <c r="K43" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L43" s="5"/>
+      <c r="L43" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M43" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>21</v>
@@ -4774,22 +4855,22 @@
     </row>
     <row r="45" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>21</v>
@@ -4815,22 +4896,22 @@
     </row>
     <row r="46" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>21</v>
@@ -4847,29 +4928,31 @@
       <c r="K46" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L46" s="5"/>
+      <c r="L46" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M46" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>21</v>
@@ -4895,25 +4978,25 @@
     </row>
     <row r="48" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="H48" s="5" t="s">
         <v>22</v>
@@ -4927,29 +5010,31 @@
       <c r="K48" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L48" s="5"/>
+      <c r="L48" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M48" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="G49" s="6" t="s">
         <v>21</v>
@@ -4966,32 +5051,34 @@
       <c r="K49" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L49" s="5"/>
+      <c r="L49" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M49" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H50" s="5" t="s">
         <v>53</v>
@@ -5014,25 +5101,25 @@
     </row>
     <row r="51" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="H51" s="5" t="s">
         <v>53</v>
@@ -5055,28 +5142,28 @@
     </row>
     <row r="52" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="G52" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I52" s="5" t="s">
         <v>23</v>
@@ -5087,29 +5174,31 @@
       <c r="K52" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L52" s="5"/>
+      <c r="L52" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M52" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G53" s="6" t="s">
         <v>21</v>
@@ -5135,22 +5224,22 @@
     </row>
     <row r="54" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G54" s="6" t="s">
         <v>21</v>
@@ -5176,22 +5265,22 @@
     </row>
     <row r="55" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="G55" s="6" t="s">
         <v>21</v>
@@ -5208,35 +5297,37 @@
       <c r="K55" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L55" s="5"/>
+      <c r="L55" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M55" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G56" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I56" s="5" t="s">
         <v>23</v>
@@ -5247,35 +5338,37 @@
       <c r="K56" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L56" s="5"/>
+      <c r="L56" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M56" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C57" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="F57" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="F57" s="6" t="s">
-        <v>277</v>
       </c>
       <c r="G57" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>23</v>
@@ -5286,35 +5379,37 @@
       <c r="K57" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L57" s="5"/>
+      <c r="L57" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M57" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="G58" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I58" s="5" t="s">
         <v>23</v>
@@ -5325,29 +5420,31 @@
       <c r="K58" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L58" s="5"/>
+      <c r="L58" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M58" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G59" s="6" t="s">
         <v>21</v>
@@ -5364,9 +5461,11 @@
       <c r="K59" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L59" s="5"/>
+      <c r="L59" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="M59" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -5398,21 +5497,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5420,10 +5519,10 @@
         <v>16</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D4" s="6"/>
     </row>
@@ -5432,10 +5531,10 @@
         <v>44</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D5" s="6"/>
     </row>
@@ -5444,10 +5543,10 @@
         <v>60</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D6" s="6"/>
     </row>
@@ -5456,13 +5555,13 @@
         <v>79</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5470,131 +5569,131 @@
         <v>84</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5602,7 +5701,7 @@
         <v>37</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>36</v>
@@ -5611,16 +5710,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5628,7 +5727,7 @@
         <v>49</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>48</v>
@@ -5637,318 +5736,318 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B46" s="10" t="n">
         <f aca="false">COUNTA('Test cases'!A5:A59)</f>
@@ -5957,7 +6056,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="9" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B47" s="10" t="n">
         <f aca="false">COUNTIF('Test cases'!I5:I59,"позитивний")</f>
@@ -5966,7 +6065,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="9" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">COUNTIF('Test cases'!I5:I59,"негативний")</f>
@@ -5975,7 +6074,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B49" s="10" t="n">
         <f aca="false">COUNTA(A4:A43)-1</f>
@@ -5984,7 +6083,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B50" s="10" t="n">
         <f aca="false">COUNTIF(C4:C43,"TC-*")</f>
@@ -5993,7 +6092,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B51" s="10" t="n">
         <f aca="false">B49-B50</f>
@@ -6002,7 +6101,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B52" s="10" t="n">
         <f aca="false">COUNTIF(A4:A43,"F-*")+COUNTIF(A4:A43,"GUI-*")</f>
@@ -6011,7 +6110,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B53" s="10" t="n">
         <f aca="false">COUNTIFS(A4:A43,"F-*",C4:C43,"TC-*")+COUNTIFS(A4:A43,"GUI-*",C4:C43,"TC-*")</f>
@@ -6048,400 +6147,400 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>422</v>
-      </c>
       <c r="G7" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>21</v>
@@ -6449,107 +6548,107 @@
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -6568,43 +6667,47 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>500</v>
-      </c>
-      <c r="B3" s="13" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
+        <v>502</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>501</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>502</v>
-      </c>
-      <c r="E3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>503</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="D3" s="12" t="s">
         <v>504</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E3" s="12" t="s">
+        <v>505</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>506</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
         <v>15</v>
       </c>
@@ -6615,13 +6718,14 @@
         <v>26</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G4" s="14"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
         <v>28</v>
       </c>
@@ -6632,13 +6736,14 @@
         <v>26</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
         <v>32</v>
       </c>
@@ -6649,13 +6754,14 @@
         <v>26</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G6" s="14"/>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
         <v>36</v>
       </c>
@@ -6665,17 +6771,20 @@
       <c r="C7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>506</v>
+      <c r="D7" s="14" t="s">
+        <v>509</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>511</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
         <v>43</v>
       </c>
@@ -6686,13 +6795,14 @@
         <v>26</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G8" s="14"/>
+    </row>
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
         <v>48</v>
       </c>
@@ -6702,17 +6812,20 @@
       <c r="C9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>509</v>
+      <c r="D9" s="14" t="s">
+        <v>513</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>514</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
         <v>54</v>
       </c>
@@ -6722,17 +6835,20 @@
       <c r="C10" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>511</v>
+      <c r="D10" s="14" t="s">
+        <v>515</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F10" s="14" t="s">
+        <v>516</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
         <v>59</v>
       </c>
@@ -6742,17 +6858,20 @@
       <c r="C11" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>513</v>
+      <c r="D11" s="14" t="s">
+        <v>517</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>518</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
         <v>64</v>
       </c>
@@ -6762,17 +6881,20 @@
       <c r="C12" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>515</v>
+      <c r="D12" s="14" t="s">
+        <v>519</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>520</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
         <v>72</v>
       </c>
@@ -6782,17 +6904,20 @@
       <c r="C13" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>517</v>
+      <c r="D13" s="14" t="s">
+        <v>521</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>522</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
         <v>78</v>
       </c>
@@ -6802,17 +6927,20 @@
       <c r="C14" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>519</v>
+      <c r="D14" s="14" t="s">
+        <v>523</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>524</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
         <v>83</v>
       </c>
@@ -6823,18 +6951,21 @@
         <v>26</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>526</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>25</v>
@@ -6842,19 +6973,22 @@
       <c r="C16" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="15" t="s">
-        <v>523</v>
+      <c r="D16" s="14" t="s">
+        <v>528</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>529</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>25</v>
@@ -6862,19 +6996,22 @@
       <c r="C17" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="15" t="s">
-        <v>511</v>
+      <c r="D17" s="14" t="s">
+        <v>515</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>530</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>25</v>
@@ -6882,19 +7019,22 @@
       <c r="C18" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="15" t="s">
-        <v>526</v>
+      <c r="D18" s="14" t="s">
+        <v>531</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>532</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>25</v>
@@ -6903,18 +7043,21 @@
         <v>26</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>533</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>25</v>
@@ -6922,19 +7065,22 @@
       <c r="C20" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="15" t="s">
-        <v>511</v>
+      <c r="D20" s="14" t="s">
+        <v>515</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>535</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>25</v>
@@ -6942,19 +7088,22 @@
       <c r="C21" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="15" t="s">
-        <v>529</v>
+      <c r="D21" s="14" t="s">
+        <v>536</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>537</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>25</v>
@@ -6962,19 +7111,22 @@
       <c r="C22" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="15" t="s">
-        <v>511</v>
+      <c r="D22" s="14" t="s">
+        <v>515</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>535</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>25</v>
@@ -6982,19 +7134,22 @@
       <c r="C23" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="15" t="s">
-        <v>511</v>
+      <c r="D23" s="14" t="s">
+        <v>515</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>535</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>25</v>
@@ -7003,15 +7158,16 @@
         <v>26</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>25</v>
@@ -7020,15 +7176,16 @@
         <v>26</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>25</v>
@@ -7037,15 +7194,16 @@
         <v>26</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E26" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>25</v>
@@ -7054,18 +7212,19 @@
         <v>26</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E27" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+      <c r="G27" s="14"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>25</v>
@@ -7074,18 +7233,19 @@
         <v>26</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+      <c r="G28" s="14"/>
+    </row>
+    <row r="29" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>25</v>
@@ -7093,19 +7253,22 @@
       <c r="C29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="15" t="s">
-        <v>532</v>
+      <c r="D29" s="14" t="s">
+        <v>539</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>540</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B30" s="14" t="s">
         <v>25</v>
@@ -7113,19 +7276,22 @@
       <c r="C30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="15" t="s">
-        <v>534</v>
+      <c r="D30" s="14" t="s">
+        <v>541</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>542</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>25</v>
@@ -7133,19 +7299,22 @@
       <c r="C31" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="15" t="s">
-        <v>536</v>
+      <c r="D31" s="14" t="s">
+        <v>543</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>544</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>25</v>
@@ -7153,19 +7322,22 @@
       <c r="C32" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="15" t="s">
-        <v>538</v>
+      <c r="D32" s="14" t="s">
+        <v>545</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>546</v>
+      </c>
+      <c r="G32" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>25</v>
@@ -7173,19 +7345,22 @@
       <c r="C33" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D33" s="15" t="s">
-        <v>540</v>
+      <c r="D33" s="14" t="s">
+        <v>547</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>548</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>25</v>
@@ -7193,19 +7368,22 @@
       <c r="C34" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="15" t="s">
-        <v>542</v>
+      <c r="D34" s="14" t="s">
+        <v>549</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>550</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>25</v>
@@ -7214,18 +7392,19 @@
         <v>26</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+      <c r="G35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>25</v>
@@ -7234,18 +7413,19 @@
         <v>26</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+      <c r="G36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>25</v>
@@ -7254,18 +7434,19 @@
         <v>26</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+      <c r="G37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>25</v>
@@ -7274,18 +7455,19 @@
         <v>26</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+      <c r="G38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>25</v>
@@ -7294,15 +7476,16 @@
         <v>26</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G39" s="14"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>25</v>
@@ -7311,15 +7494,16 @@
         <v>26</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E40" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G40" s="14"/>
+    </row>
+    <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>25</v>
@@ -7327,19 +7511,22 @@
       <c r="C41" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D41" s="15" t="s">
-        <v>544</v>
+      <c r="D41" s="14" t="s">
+        <v>551</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>552</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>25</v>
@@ -7347,19 +7534,22 @@
       <c r="C42" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D42" s="15" t="s">
-        <v>546</v>
+      <c r="D42" s="14" t="s">
+        <v>553</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>554</v>
+      </c>
+      <c r="G42" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="14" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>25</v>
@@ -7368,15 +7558,16 @@
         <v>26</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G43" s="14"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>25</v>
@@ -7385,15 +7576,16 @@
         <v>26</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G44" s="14"/>
+    </row>
+    <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>25</v>
@@ -7401,19 +7593,22 @@
       <c r="C45" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D45" s="15" t="s">
-        <v>548</v>
+      <c r="D45" s="14" t="s">
+        <v>555</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>556</v>
+      </c>
+      <c r="G45" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>25</v>
@@ -7422,15 +7617,16 @@
         <v>26</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="47" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G46" s="14"/>
+    </row>
+    <row r="47" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>25</v>
@@ -7438,19 +7634,22 @@
       <c r="C47" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D47" s="15" t="s">
-        <v>550</v>
+      <c r="D47" s="14" t="s">
+        <v>557</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>558</v>
+      </c>
+      <c r="G47" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>25</v>
@@ -7458,19 +7657,22 @@
       <c r="C48" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D48" s="15" t="s">
-        <v>552</v>
+      <c r="D48" s="14" t="s">
+        <v>559</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>560</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>25</v>
@@ -7479,15 +7681,16 @@
         <v>26</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E49" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G49" s="14"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B50" s="14" t="s">
         <v>25</v>
@@ -7496,15 +7699,16 @@
         <v>26</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G50" s="14"/>
+    </row>
+    <row r="51" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B51" s="14" t="s">
         <v>25</v>
@@ -7512,19 +7716,22 @@
       <c r="C51" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D51" s="15" t="s">
-        <v>554</v>
+      <c r="D51" s="14" t="s">
+        <v>561</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>562</v>
+      </c>
+      <c r="G51" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B52" s="14" t="s">
         <v>25</v>
@@ -7533,15 +7740,16 @@
         <v>26</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E52" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G52" s="14"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>25</v>
@@ -7550,15 +7758,16 @@
         <v>26</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E53" s="14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="54" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G53" s="14"/>
+    </row>
+    <row r="54" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B54" s="14" t="s">
         <v>25</v>
@@ -7566,19 +7775,22 @@
       <c r="C54" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D54" s="15" t="s">
-        <v>556</v>
+      <c r="D54" s="14" t="s">
+        <v>563</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>564</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>25</v>
@@ -7586,19 +7798,22 @@
       <c r="C55" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D55" s="15" t="s">
-        <v>558</v>
+      <c r="D55" s="14" t="s">
+        <v>565</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>566</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B56" s="14" t="s">
         <v>25</v>
@@ -7606,19 +7821,22 @@
       <c r="C56" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D56" s="15" t="s">
-        <v>560</v>
+      <c r="D56" s="14" t="s">
+        <v>567</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>568</v>
+      </c>
+      <c r="G56" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>25</v>
@@ -7626,19 +7844,22 @@
       <c r="C57" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D57" s="15" t="s">
-        <v>511</v>
+      <c r="D57" s="14" t="s">
+        <v>515</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F57" s="14" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>535</v>
+      </c>
+      <c r="G57" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B58" s="14" t="s">
         <v>25</v>
@@ -7646,51 +7867,54 @@
       <c r="C58" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D58" s="15" t="s">
-        <v>562</v>
+      <c r="D58" s="14" t="s">
+        <v>569</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F58" s="14" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>570</v>
+      </c>
+      <c r="G58" s="14" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="16" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>

</xml_diff>